<commit_message>
Import customer emails as contacts
</commit_message>
<xml_diff>
--- a/docs/templates/base-clientes-modelo.xlsx
+++ b/docs/templates/base-clientes-modelo.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H5"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,15 +410,18 @@
         <v>Nome Fantasia</v>
       </c>
       <c r="D1" t="str">
+        <v>Email</v>
+      </c>
+      <c r="E1" t="str">
         <v>Endereco</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>Cidade</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>UF</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>CEP</v>
       </c>
     </row>
@@ -433,67 +436,102 @@
         <v>ALPHA</v>
       </c>
       <c r="D2" t="str">
+        <v>OPERACIONAL@ALPHA.COM.BR</v>
+      </c>
+      <c r="E2" t="str">
         <v>RUA EXEMPLO 100, SALA 1</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>VITORIA</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>ES</v>
       </c>
-      <c r="G2" t="str">
+      <c r="H2" t="str">
         <v>29000000</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>11222333000144</v>
+        <v>12345678000195</v>
       </c>
       <c r="B3" t="str">
-        <v>IMPORTADORA GAMMA LTDA</v>
+        <v>IMPORTADORA ALPHA LTDA</v>
       </c>
       <c r="C3" t="str">
-        <v>GAMMA</v>
+        <v>ALPHA</v>
       </c>
       <c r="D3" t="str">
-        <v>AVENIDA CENTRAL 200</v>
+        <v>FINANCEIRO@ALPHA.COM.BR</v>
       </c>
       <c r="E3" t="str">
-        <v>SALVADOR</v>
+        <v>RUA EXEMPLO 100, SALA 1</v>
       </c>
       <c r="F3" t="str">
-        <v>BA</v>
+        <v>VITORIA</v>
       </c>
       <c r="G3" t="str">
-        <v>40000000</v>
+        <v>ES</v>
+      </c>
+      <c r="H3" t="str">
+        <v>29000000</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v>11222333000144</v>
+      </c>
+      <c r="B4" t="str">
+        <v>IMPORTADORA GAMMA LTDA</v>
+      </c>
+      <c r="C4" t="str">
+        <v>GAMMA</v>
+      </c>
+      <c r="D4" t="str">
+        <v>IMPORTACAO@GAMMA.COM.BR</v>
+      </c>
+      <c r="E4" t="str">
+        <v>AVENIDA CENTRAL 200</v>
+      </c>
+      <c r="F4" t="str">
+        <v>SALVADOR</v>
+      </c>
+      <c r="G4" t="str">
+        <v>BA</v>
+      </c>
+      <c r="H4" t="str">
+        <v>40000000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
         <v>99888777000166</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B5" t="str">
         <v>LOGISTICA DELTA COMERCIO EXTERIOR LTDA</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C5" t="str">
         <v>DELTA</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D5" t="str">
+        <v>CONTATO@DELTA.COM.BR</v>
+      </c>
+      <c r="E5" t="str">
         <v>RUA DO PORTO 50</v>
       </c>
-      <c r="E4" t="str">
+      <c r="F5" t="str">
         <v>SANTOS</v>
       </c>
-      <c r="F4" t="str">
+      <c r="G5" t="str">
         <v>SP</v>
       </c>
-      <c r="G4" t="str">
+      <c r="H5" t="str">
         <v>11000000</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H5"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>